<commit_message>
agregadas las variables para alumnos inscritos en la seccion
</commit_message>
<xml_diff>
--- a/backend/templates/resumenFinal_template_ - Copy.xlsx
+++ b/backend/templates/resumenFinal_template_ - Copy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JavierWorkSpace\BatallaProject\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F01CF8A-397D-4A6A-9F80-F27A15C6D7E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2664C511-0725-40E0-815A-24EE9C68D5B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{299BAFB4-AE58-4015-B36E-D7CD92F1B4DD}"/>
   </bookViews>
@@ -713,6 +713,15 @@
     <definedName name="subj_7">'1er Año'!$T$15</definedName>
     <definedName name="subj_8">'1er Año'!$U$15</definedName>
     <definedName name="subj_9">'1er Año'!$V$15</definedName>
+    <definedName name="subj_count_1">'1er Año'!$N$51</definedName>
+    <definedName name="subj_count_2">'1er Año'!$O$51</definedName>
+    <definedName name="subj_count_3">'1er Año'!$P$51</definedName>
+    <definedName name="subj_count_4">'1er Año'!$Q$51</definedName>
+    <definedName name="subj_count_5">'1er Año'!$R$51</definedName>
+    <definedName name="subj_count_6">'1er Año'!$S$51</definedName>
+    <definedName name="subj_count_7">'1er Año'!$T$51</definedName>
+    <definedName name="subj_count_8">'1er Año'!$U$51</definedName>
+    <definedName name="subj_count_9">'1er Año'!$V$51</definedName>
     <definedName name="subj_failed_1">'1er Año'!$N$54</definedName>
     <definedName name="subj_failed_2">'1er Año'!$O$54</definedName>
     <definedName name="subj_failed_3">'1er Año'!$P$54</definedName>
@@ -722,6 +731,35 @@
     <definedName name="subj_failed_7">'1er Año'!$T$54</definedName>
     <definedName name="subj_failed_8">'1er Año'!$U$54</definedName>
     <definedName name="subj_failed_9">'1er Año'!$V$54</definedName>
+    <definedName name="subj_failed_i6">'1er Año'!$S$54</definedName>
+    <definedName name="subj_passed_1">'1er Año'!$N$53</definedName>
+    <definedName name="subj_passed_2">'1er Año'!$O$53</definedName>
+    <definedName name="subj_passed_3">'1er Año'!$P$53</definedName>
+    <definedName name="subj_passed_4">'1er Año'!$Q$53</definedName>
+    <definedName name="subj_passed_5">'1er Año'!$R$53</definedName>
+    <definedName name="subj_passed_6">'1er Año'!$S$53</definedName>
+    <definedName name="subj_passed_7">'1er Año'!$T$53</definedName>
+    <definedName name="subj_passed_8">'1er Año'!$U$53</definedName>
+    <definedName name="subj_passed_9">'1er Año'!$V$53</definedName>
+    <definedName name="subj_passed_i4">'1er Año'!$Q$53</definedName>
+    <definedName name="subj_unenrolled_1">'1er Año'!$N$55</definedName>
+    <definedName name="subj_unenrolled_2">'1er Año'!$O$55</definedName>
+    <definedName name="subj_unenrolled_3">'1er Año'!$P$55</definedName>
+    <definedName name="subj_unenrolled_4">'1er Año'!$Q$55</definedName>
+    <definedName name="subj_unenrolled_5">'1er Año'!$R$55</definedName>
+    <definedName name="subj_unenrolled_6">'1er Año'!$S$55</definedName>
+    <definedName name="subj_unenrolled_7">'1er Año'!$T$55</definedName>
+    <definedName name="subj_unenrolled_8">'1er Año'!$U$55</definedName>
+    <definedName name="subj_unenrolled_9">'1er Año'!$V$55</definedName>
+    <definedName name="subj_zero_1">'1er Año'!$N$52</definedName>
+    <definedName name="subj_zero_2">'1er Año'!$O$52</definedName>
+    <definedName name="subj_zero_3">'1er Año'!$P$52</definedName>
+    <definedName name="subj_zero_4">'1er Año'!$Q$52</definedName>
+    <definedName name="subj_zero_5">'1er Año'!$R$52</definedName>
+    <definedName name="subj_zero_6">'1er Año'!$S$52</definedName>
+    <definedName name="subj_zero_7">'1er Año'!$T$52</definedName>
+    <definedName name="subj_zero_8">'1er Año'!$U$52</definedName>
+    <definedName name="subj_zero_9">'1er Año'!$V$52</definedName>
     <definedName name="subjname_1">'1er Año'!$C$58</definedName>
     <definedName name="subjname_2">'1er Año'!$C$59</definedName>
     <definedName name="subjname_3">'1er Año'!$C$60</definedName>

</xml_diff>